<commit_message>
Refactor workbook structure: replace milestones with dimensions
- Updated the workbook README to reflect changes from milestones to dimensions.
- Modified the workbook validator to validate dimension-related fields instead of milestone fields.
- Adjusted the setup script to build questions with dimension attributes.
- Changed evidence explorer and milestone board components to reference dimensions instead of milestones.
- Updated community feedback components to handle dimensions and questions.
- Created new community form and snapshot components for public input on dimensions.
- Added community suggestions data structure and utility functions for building community links.
</commit_message>
<xml_diff>
--- a/content/workbook/AGI benchmark mapping.xlsx
+++ b/content/workbook/AGI benchmark mapping.xlsx
@@ -1,36 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D82DFC-77A0-4665-9158-E192DBFE3D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-14295" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Questions" sheetId="1" r:id="rId1"/>
-    <sheet name="Evidence" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Questions" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Evidence" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="426">
   <si>
-    <t>milestone_id</t>
-  </si>
-  <si>
-    <t>milestone_title</t>
-  </si>
-  <si>
-    <t>milestone_description</t>
-  </si>
-  <si>
-    <t>milestone_category</t>
-  </si>
-  <si>
-    <t>milestone_sort_order</t>
+    <t>dimension_id</t>
+  </si>
+  <si>
+    <t>dimension_title</t>
+  </si>
+  <si>
+    <t>dimension_description</t>
+  </si>
+  <si>
+    <t>dimension_category</t>
+  </si>
+  <si>
+    <t>dimension_sort_order</t>
   </si>
   <si>
     <t>question_id</t>
@@ -1299,20 +1295,18 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FF22313F"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1754,18 +1748,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T76"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
-    <col min="2" max="2" width="77.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="154.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="48" style="2" customWidth="1"/>
     <col min="4" max="4" width="22" style="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" customWidth="1"/>
     <col min="6" max="6" width="28" style="1" customWidth="1"/>
     <col min="7" max="7" width="16" style="1" customWidth="1"/>
-    <col min="8" max="8" width="65.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44" style="2" customWidth="1"/>
     <col min="9" max="9" width="52" style="2" customWidth="1"/>
     <col min="10" max="11" width="16" style="1" customWidth="1"/>
     <col min="12" max="12" width="52" style="2" customWidth="1"/>
@@ -1777,7 +1771,7 @@
     <col min="19" max="20" width="34" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1839,7 +1833,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>20</v>
       </c>
@@ -1901,7 +1895,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>20</v>
       </c>
@@ -1963,7 +1957,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>20</v>
       </c>
@@ -2025,7 +2019,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
@@ -2087,7 +2081,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>20</v>
       </c>
@@ -2149,7 +2143,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>53</v>
       </c>
@@ -2211,7 +2205,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>53</v>
       </c>
@@ -2273,7 +2267,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>53</v>
       </c>
@@ -2335,7 +2329,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>53</v>
       </c>
@@ -2397,7 +2391,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>53</v>
       </c>
@@ -2459,7 +2453,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>79</v>
       </c>
@@ -2521,7 +2515,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>79</v>
       </c>
@@ -2583,7 +2577,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>79</v>
       </c>
@@ -2645,7 +2639,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>79</v>
       </c>
@@ -2707,7 +2701,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>79</v>
       </c>
@@ -2769,7 +2763,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>107</v>
       </c>
@@ -2831,7 +2825,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>107</v>
       </c>
@@ -2893,7 +2887,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>107</v>
       </c>
@@ -2955,7 +2949,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>107</v>
       </c>
@@ -3017,7 +3011,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>107</v>
       </c>
@@ -3079,7 +3073,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>135</v>
       </c>
@@ -3141,7 +3135,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>135</v>
       </c>
@@ -3203,7 +3197,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>135</v>
       </c>
@@ -3265,7 +3259,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>135</v>
       </c>
@@ -3327,7 +3321,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>135</v>
       </c>
@@ -3389,7 +3383,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>161</v>
       </c>
@@ -3451,7 +3445,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>161</v>
       </c>
@@ -3513,7 +3507,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>161</v>
       </c>
@@ -3575,7 +3569,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>161</v>
       </c>
@@ -3637,7 +3631,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>161</v>
       </c>
@@ -3699,7 +3693,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>189</v>
       </c>
@@ -3761,7 +3755,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>189</v>
       </c>
@@ -3823,7 +3817,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>189</v>
       </c>
@@ -3885,7 +3879,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>189</v>
       </c>
@@ -3947,7 +3941,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>189</v>
       </c>
@@ -4009,7 +4003,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>213</v>
       </c>
@@ -4071,7 +4065,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>213</v>
       </c>
@@ -4133,7 +4127,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>213</v>
       </c>
@@ -4195,7 +4189,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>213</v>
       </c>
@@ -4257,7 +4251,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
         <v>213</v>
       </c>
@@ -4319,7 +4313,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
         <v>238</v>
       </c>
@@ -4381,7 +4375,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>238</v>
       </c>
@@ -4443,7 +4437,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>238</v>
       </c>
@@ -4505,7 +4499,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>238</v>
       </c>
@@ -4567,7 +4561,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>238</v>
       </c>
@@ -4629,7 +4623,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>263</v>
       </c>
@@ -4691,7 +4685,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>263</v>
       </c>
@@ -4753,7 +4747,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>263</v>
       </c>
@@ -4815,7 +4809,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="50" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>263</v>
       </c>
@@ -4877,7 +4871,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>263</v>
       </c>
@@ -4939,7 +4933,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="52" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>287</v>
       </c>
@@ -5001,7 +4995,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>287</v>
       </c>
@@ -5063,7 +5057,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>287</v>
       </c>
@@ -5125,7 +5119,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>287</v>
       </c>
@@ -5187,7 +5181,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>287</v>
       </c>
@@ -5249,7 +5243,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="57" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>312</v>
       </c>
@@ -5311,7 +5305,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>312</v>
       </c>
@@ -5373,7 +5367,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
         <v>312</v>
       </c>
@@ -5435,7 +5429,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="60" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
         <v>312</v>
       </c>
@@ -5497,7 +5491,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>312</v>
       </c>
@@ -5559,7 +5553,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
         <v>337</v>
       </c>
@@ -5621,7 +5615,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>337</v>
       </c>
@@ -5683,7 +5677,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
         <v>337</v>
       </c>
@@ -5745,7 +5739,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="65" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
         <v>337</v>
       </c>
@@ -5807,7 +5801,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>337</v>
       </c>
@@ -5869,7 +5863,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="67" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
         <v>363</v>
       </c>
@@ -5931,7 +5925,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="68" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
         <v>363</v>
       </c>
@@ -5993,7 +5987,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="69" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
         <v>363</v>
       </c>
@@ -6055,7 +6049,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
         <v>363</v>
       </c>
@@ -6117,7 +6111,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="71" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
         <v>363</v>
       </c>
@@ -6179,7 +6173,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
         <v>387</v>
       </c>
@@ -6241,7 +6235,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
         <v>387</v>
       </c>
@@ -6303,7 +6297,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="74" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>387</v>
       </c>
@@ -6365,7 +6359,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="75" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
         <v>387</v>
       </c>
@@ -6427,7 +6421,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="76" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" ht="22" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>387</v>
       </c>
@@ -6490,24 +6484,24 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:T1"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="J2:J500" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="J2:J500">
       <formula1>"unassessed,not_met,in_progress,met"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="K2:K500" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="K2:K500">
       <formula1>"unassessed,low,medium,high"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
     <col min="2" max="2" width="28" style="1" customWidth="1"/>
@@ -6525,7 +6519,7 @@
     <col min="14" max="14" width="12" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>413</v>
       </c>
@@ -6570,16 +6564,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:N1"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="D2:D500" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="D2:D500">
       <formula1>"benchmark,leaderboard,research_paper,news,implementation"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="N2:N500" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of the dropdown values." sqref="N2:N500">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>